<commit_message>
Actualizar maestros de proveedores vía Telegram (4944 nuevos, 0 corregidos)
Enviado por Telegram, aplicado sin revisión.
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5035"/>
+  <dimension ref="A1:B5049"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -40679,9 +40679,121 @@
         <v>SUC. DE EMILIO GROSS SRL</v>
       </c>
     </row>
+    <row r="5036">
+      <c r="A5036" t="str">
+        <v>30709577456</v>
+      </c>
+      <c r="B5036" t="str">
+        <v>OPERADORA RIVENDELL SA</v>
+      </c>
+    </row>
+    <row r="5037">
+      <c r="A5037" t="str">
+        <v>30718973755</v>
+      </c>
+      <c r="B5037" t="str">
+        <v>CALA LIBRERIA SOC. CAPITLO 1</v>
+      </c>
+    </row>
+    <row r="5038">
+      <c r="A5038" t="str">
+        <v>20226976354</v>
+      </c>
+      <c r="B5038" t="str">
+        <v>CARRIZO MARIO</v>
+      </c>
+    </row>
+    <row r="5039">
+      <c r="A5039" t="str">
+        <v>27242644544</v>
+      </c>
+      <c r="B5039" t="str">
+        <v>ROMAN FERNANDA M. EUGENIA</v>
+      </c>
+    </row>
+    <row r="5040">
+      <c r="A5040" t="str">
+        <v>33707955959</v>
+      </c>
+      <c r="B5040" t="str">
+        <v>DACHSER SA</v>
+      </c>
+    </row>
+    <row r="5041">
+      <c r="A5041" t="str">
+        <v>30670840014</v>
+      </c>
+      <c r="B5041" t="str">
+        <v>VETERINARIA HERNANDEZ SRL</v>
+      </c>
+    </row>
+    <row r="5042">
+      <c r="A5042" t="str">
+        <v>23374258869</v>
+      </c>
+      <c r="B5042" t="str">
+        <v>LAMAISON NICOLAS</v>
+      </c>
+    </row>
+    <row r="5043">
+      <c r="A5043" t="str">
+        <v>30708717262</v>
+      </c>
+      <c r="B5043" t="str">
+        <v>ITAPE SA</v>
+      </c>
+    </row>
+    <row r="5044">
+      <c r="A5044" t="str">
+        <v>27343793478</v>
+      </c>
+      <c r="B5044" t="str">
+        <v>ESQUIVEL SOFIA BELEN</v>
+      </c>
+    </row>
+    <row r="5045">
+      <c r="A5045" t="str">
+        <v>20297695615</v>
+      </c>
+      <c r="B5045" t="str">
+        <v>MONRROI HECTOR PAOLO</v>
+      </c>
+    </row>
+    <row r="5046">
+      <c r="A5046" t="str">
+        <v>30651802063</v>
+      </c>
+      <c r="B5046" t="str">
+        <v>AGROAR MAQUINAS AGRICOLAS</v>
+      </c>
+    </row>
+    <row r="5047">
+      <c r="A5047" t="str">
+        <v>27354405909</v>
+      </c>
+      <c r="B5047" t="str">
+        <v>MEDINA LEANDRO GABRIEL</v>
+      </c>
+    </row>
+    <row r="5048">
+      <c r="A5048" t="str">
+        <v>23139936183</v>
+      </c>
+      <c r="B5048" t="str">
+        <v>BENITO ALBERTO RUBEN</v>
+      </c>
+    </row>
+    <row r="5049">
+      <c r="A5049" t="str">
+        <v>20317692944</v>
+      </c>
+      <c r="B5049" t="str">
+        <v>ABRIL JUAN CRUZ</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5035"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5049"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar maestros de proveedores vía Telegram (30 nuevos, 2 corregidos)
Enviado por Telegram, aplicado sin revisión.
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5049"/>
+  <dimension ref="A1:B5064"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -34148,7 +34148,7 @@
         <v>30-71855351-9</v>
       </c>
       <c r="B4219" t="str">
-        <v>AUTOP PROV AP 01 BRIG GRAL ESTAN</v>
+        <v>AUTOPISTA PROVINCIAL AP 01</v>
       </c>
     </row>
     <row r="4220">
@@ -40791,9 +40791,129 @@
         <v>ABRIL JUAN CRUZ</v>
       </c>
     </row>
+    <row r="5050">
+      <c r="A5050" t="str">
+        <v>30715310283</v>
+      </c>
+      <c r="B5050" t="str">
+        <v>GASRRONI S.R.L.</v>
+      </c>
+    </row>
+    <row r="5051">
+      <c r="A5051" t="str">
+        <v>20206686880</v>
+      </c>
+      <c r="B5051" t="str">
+        <v>RIOS RAMON HERMENEGILDO</v>
+      </c>
+    </row>
+    <row r="5052">
+      <c r="A5052" t="str">
+        <v>30719454190</v>
+      </c>
+      <c r="B5052" t="str">
+        <v>RUTAS SUR ATLANTICO SA</v>
+      </c>
+    </row>
+    <row r="5053">
+      <c r="A5053" t="str">
+        <v>30719244331</v>
+      </c>
+      <c r="B5053" t="str">
+        <v>CONEXION ALTO DELTA</v>
+      </c>
+    </row>
+    <row r="5054">
+      <c r="A5054" t="str">
+        <v>30719231191</v>
+      </c>
+      <c r="B5054" t="str">
+        <v>AUTOVIA DEL MERCOSUR SAU</v>
+      </c>
+    </row>
+    <row r="5055">
+      <c r="A5055" t="str">
+        <v>30719461413</v>
+      </c>
+      <c r="B5055" t="str">
+        <v>CORREDOR VIAL 5 SAU</v>
+      </c>
+    </row>
+    <row r="5056">
+      <c r="A5056" t="str">
+        <v>20206154625</v>
+      </c>
+      <c r="B5056" t="str">
+        <v>GIBEZZI CARLOS ALBERTO</v>
+      </c>
+    </row>
+    <row r="5057">
+      <c r="A5057" t="str">
+        <v>20269739755</v>
+      </c>
+      <c r="B5057" t="str">
+        <v>BERTANI MAURICIO</v>
+      </c>
+    </row>
+    <row r="5058">
+      <c r="A5058" t="str">
+        <v>20293758876</v>
+      </c>
+      <c r="B5058" t="str">
+        <v>_x0002_LANZA JORGE DANIEL</v>
+      </c>
+    </row>
+    <row r="5059">
+      <c r="A5059" t="str">
+        <v>23169927634</v>
+      </c>
+      <c r="B5059" t="str">
+        <v>REVOREDO M. CECILIA</v>
+      </c>
+    </row>
+    <row r="5060">
+      <c r="A5060" t="str">
+        <v>30503095846</v>
+      </c>
+      <c r="B5060" t="str">
+        <v>FRANCAVILLA HNOS SA</v>
+      </c>
+    </row>
+    <row r="5061">
+      <c r="A5061" t="str">
+        <v>27238592483</v>
+      </c>
+      <c r="B5061" t="str">
+        <v>LUGONES ALEJANDRA</v>
+      </c>
+    </row>
+    <row r="5062">
+      <c r="A5062" t="str">
+        <v>30712161953</v>
+      </c>
+      <c r="B5062" t="str">
+        <v>DHM INDUSTRIA SA</v>
+      </c>
+    </row>
+    <row r="5063">
+      <c r="A5063" t="str">
+        <v>30650637638</v>
+      </c>
+      <c r="B5063" t="str">
+        <v>SOC. ARGENTINA DE APICULTORES</v>
+      </c>
+    </row>
+    <row r="5064">
+      <c r="A5064" t="str">
+        <v>30582215703</v>
+      </c>
+      <c r="B5064" t="str">
+        <v>CVC SA</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5049"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5064"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar maestros de proveedores vía Telegram (14 nuevos, 2 corregidos)
Enviado por Telegram, aplicado sin revisión.
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5064"/>
+  <dimension ref="A1:B5071"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3700,7 +3700,7 @@
         <v>30-70786712-0</v>
       </c>
       <c r="B413" t="str">
-        <v>LOGISTICA GAMMA S.A.</v>
+        <v>GAMMA  LOGISTICA</v>
       </c>
     </row>
     <row r="414">
@@ -40911,9 +40911,65 @@
         <v>CVC SA</v>
       </c>
     </row>
+    <row r="5065">
+      <c r="A5065" t="str">
+        <v>30715666002</v>
+      </c>
+      <c r="B5065" t="str">
+        <v>NAYAR DANIEL  Y NAYAR  JULIAN</v>
+      </c>
+    </row>
+    <row r="5066">
+      <c r="A5066" t="str">
+        <v>30711923272</v>
+      </c>
+      <c r="B5066" t="str">
+        <v>SCC TRADING SRL</v>
+      </c>
+    </row>
+    <row r="5067">
+      <c r="A5067" t="str">
+        <v>27214146229</v>
+      </c>
+      <c r="B5067" t="str">
+        <v>DELBONO ANDREA SUSANA</v>
+      </c>
+    </row>
+    <row r="5068">
+      <c r="A5068" t="str">
+        <v>20278555896</v>
+      </c>
+      <c r="B5068" t="str">
+        <v>BIROCCIO NICOLAS</v>
+      </c>
+    </row>
+    <row r="5069">
+      <c r="A5069" t="str">
+        <v>20240801214</v>
+      </c>
+      <c r="B5069" t="str">
+        <v>SCARDINI CLAUDIO ALFREDO</v>
+      </c>
+    </row>
+    <row r="5070">
+      <c r="A5070" t="str">
+        <v>30719215986</v>
+      </c>
+      <c r="B5070" t="str">
+        <v>CENTRO DE SERVICIOS GUALEGUAYCHU SRL</v>
+      </c>
+    </row>
+    <row r="5071">
+      <c r="A5071" t="str">
+        <v>20284529163</v>
+      </c>
+      <c r="B5071" t="str">
+        <v>ZARLENGA RODRIGO</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5064"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5071"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>